<commit_message>
❌ Eliminazione Massiva di 1 Assegni effettuata da Ufficio
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,42 +457,6 @@
           <t>DATA_VERSAMENTO</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>12/10/2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>UFFICIO_CENTRALE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>9387540941</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>2312</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>In Portafoglio</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 900 - Locale: EA560077165A - AL BARILOTT
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,42 @@
           <t>DATA_VERSAMENTO</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EA560077165A - AL BARILOTT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>7984</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 0568896690 - Locale: EA560061915O - CAFFE' STAZIONE
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,6 +493,42 @@
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EA560061915O - CAFFE' STAZIONE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0568896690</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2912</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 00000909 - Locale: EA600008487R - BAR ITALO
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,42 @@
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EA600008487R - BAR ITALO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>00000909</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>14386</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 9387540941-12 - Locale: EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -1,106 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuela.arigoni\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5181BC-66B7-4AB5-9AE5-114ADAFCAEEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-23415" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
-  <si>
-    <t>ESATTORE</t>
-  </si>
-  <si>
-    <t>LOCALE</t>
-  </si>
-  <si>
-    <t>NUMERO_ASSEGNO</t>
-  </si>
-  <si>
-    <t>IMPORTO</t>
-  </si>
-  <si>
-    <t>STATO_VERSAMENTO</t>
-  </si>
-  <si>
-    <t>12/10/2026</t>
-  </si>
-  <si>
-    <t>MAURIZIO ADONI</t>
-  </si>
-  <si>
-    <t>EA560077165A - AL BARILOTT</t>
-  </si>
-  <si>
-    <t>900</t>
-  </si>
-  <si>
-    <t>13/10/2026</t>
-  </si>
-  <si>
-    <t>In Portafoglio</t>
-  </si>
-  <si>
-    <t>EA560061915O - CAFFE' STAZIONE</t>
-  </si>
-  <si>
-    <t>0568896690</t>
-  </si>
-  <si>
-    <t>20/10/2026</t>
-  </si>
-  <si>
-    <t>EA600008487R - BAR ITALO</t>
-  </si>
-  <si>
-    <t>00000909</t>
-  </si>
-  <si>
-    <t>DATA_ASSEGNO</t>
-  </si>
-  <si>
-    <t>DATA_INCASSO</t>
-  </si>
-  <si>
-    <t>DATA_REGISTRAZIONE</t>
-  </si>
-  <si>
-    <t>06/10/2026</t>
-  </si>
-  <si>
-    <t>01/10/2026</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -118,24 +46,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -423,122 +408,214 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DATA_REGISTRAZIONE</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ESATTORE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>LOCALE</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NUMERO_ASSEGNO</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>IMPORTO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>DATA_ASSEGNO</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>DATA_INCASSO</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>STATO_VERSAMENTO</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EA560077165A - AL BARILOTT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>7984</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>10</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EA560061915O - CAFFE' STAZIONE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0568896690</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>2912</v>
       </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>10</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EA600008487R - BAR ITALO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>00000909</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>14386</v>
       </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>10</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MANUELA ARIGONI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>9387540941-12</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2312</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 0022670857
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A0A0A0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A0A0A0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A0A0A0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A0A0A0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,206 +432,256 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EA560077165A - AL BARILOTT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>7984</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>2912</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EA600008487R - BAR ITALO</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>00000909</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>14386</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>01/10/2026</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>2312</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>LUCA ARABENI</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>EA110075598A - NON SOLO FUMO</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>0022670857</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3579</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 902
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -687,6 +687,46 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>EA600145288K - SALA SLOT VLT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>902</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>5525</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 [Pulizia Campi Doppi]
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -63,9 +60,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,16 +430,6 @@
   </sheetPr>
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -488,240 +474,240 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>EA560077165A - AL BARILOTT</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>7984</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>In Portafoglio</t>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Versato OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>2912</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>EA600008487R - BAR ITALO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>00000909</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>14386</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>01/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>In Portafoglio</t>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Versato OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>2312</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>3579</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>5525</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 0112120453
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,8 +63,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -428,8 +432,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -474,160 +488,200 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>UFFICIO_CENTRALE</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>EA110017705R - BAR PIT STOP</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>0112120453</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>4836</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 0967584051
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -432,12 +432,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -767,6 +767,46 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>RICCARDO ROSSO</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>EA590017319S - TABACCHERIA RICEVITORIA VISENTINI PAOLO</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0967584051</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1717</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 4593
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -807,6 +807,46 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SIMONE CEREA</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>EA570032568A - AISHA'S CAFE'</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>4593</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>5147</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 12p
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,8 +63,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -428,8 +432,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -474,320 +488,360 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" s="1" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" s="1" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" s="1" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" s="1" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" s="1" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MAURIZIO ADONI</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>EA600145289K - HAVANA SALA SLOT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>12p</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>14843</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
📝 Rettifica Amministrativa Assegno N. 120
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,28 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00A0A0A0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00A0A0A0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A0A0A0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A0A0A0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,414 +415,404 @@
   </sheetPr>
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>EA600145289K - HAVANA SALA SLOT</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>12p</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
         <v>14843</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 00000911
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A0A0A0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A0A0A0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A0A0A0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A0A0A0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,406 +432,456 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>EA600145289K - HAVANA SALA SLOT</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>14843</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>UFFICIO_CENTRALE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>EA570011433R - ULTIMA PRIMA BAR TABACCHI</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>00000911</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>2466</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
📝 Rettifica Amministrativa Assegno N. 00000911
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,28 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00A0A0A0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00A0A0A0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A0A0A0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A0A0A0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,454 +415,444 @@
   </sheetPr>
   <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>EA600145289K - HAVANA SALA SLOT</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" t="n">
         <v>14843</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>UFFICIO_CENTRALE</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SIMONE CEREA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>EA570011433R - ULTIMA PRIMA BAR TABACCHI</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>00000911</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" t="n">
         <v>2466</v>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 3823772224
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A0A0A0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A0A0A0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A0A0A0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A0A0A0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,446 +432,496 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>EA600145289K - HAVANA SALA SLOT</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>14843</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>EA570011433R - ULTIMA PRIMA BAR TABACCHI</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>00000911</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>2466</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>RICCARDO ROSSO</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>EA230020700R - BAR QUINTAVALLE</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>3823772224</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>34249</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 9389348651-07
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -927,6 +927,46 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SIMONE CEREA</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>EA570047109R - BAR SPORT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>9389348651-07</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1056</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🏦 Inserimento Assegno 9389348652
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -967,6 +967,46 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SIMONE CEREA</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>EA570047109R - BAR SPORT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>9389348652</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1056</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>In Portafoglio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 [Controllo Notturno] Aggiornamento Stati Assegni
</commit_message>
<xml_diff>
--- a/registro_assegni.xlsx
+++ b/registro_assegni.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,28 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00A0A0A0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00A0A0A0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00A0A0A0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00A0A0A0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,574 +415,564 @@
   </sheetPr>
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>DATA_REGISTRAZIONE</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ESATTORE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>LOCALE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>NUMERO_ASSEGNO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>IMPORTO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DATA_ASSEGNO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>DATA_INCASSO</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>STATO_VERSAMENTO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>EA560061915O - CAFFE' STAZIONE</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>0568896690</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>2912</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>MANUELA ARIGONI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>EA090004379E - FRASH S.A.S. DI FRASCERRA MATTIA E C.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>9387540941-12</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" t="n">
         <v>2312</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>08/10/2026</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>EA110075598A - NON SOLO FUMO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>0022670857</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>3579</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>22/10/2026</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>EA600145288K - SALA SLOT VLT</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>902</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" t="n">
         <v>5525</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>13/10/2026</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>In Portafoglio</t>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Versato OK</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>EA110017705R - BAR PIT STOP</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>0112120453</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" t="n">
         <v>4836</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>SAVERIO BIANCO</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>EA110067815M - GREEN CAFE'</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>00000912</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" t="n">
         <v>2056</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>LUCA ARABENI</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>EA110071158R - BAR TABACCHERIA EDEN</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>9024634327-07</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" t="n">
         <v>2000</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>03/11/2026</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>EA570032568A - AISHA'S CAFE'</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>4593</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" t="n">
         <v>5147</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>MAURIZIO ADONI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>EA600145289K - HAVANA SALA SLOT</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" t="n">
         <v>14843</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>23/10/2026</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>15/10/2026</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>EA570011433R - ULTIMA PRIMA BAR TABACCHI</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>00000911</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" t="n">
         <v>2466</v>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>RICCARDO ROSSO</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>EA230020700R - BAR QUINTAVALLE</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>3823772224</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" t="n">
         <v>34249</v>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>30/10/2026</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>EA570047109R - BAR SPORT</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>9389348651-07</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" t="n">
         <v>1056</v>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>20/10/2026</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>SIMONE CEREA</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>EA570047109R - BAR SPORT</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>9389348652</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" t="n">
         <v>1056</v>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>27/10/2026</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>In Portafoglio</t>
         </is>

</xml_diff>